<commit_message>
docs: update production verification evidence
</commit_message>
<xml_diff>
--- a/outputs/01a08555-6f7c-7911-8b1c-f21a1a8ea9c3/COSMIC_PULSE_헌법_준수_테스트_근거.xlsx
+++ b/outputs/01a08555-6f7c-7911-8b1c-f21a1a8ea9c3/COSMIC_PULSE_헌법_준수_테스트_근거.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R869417fb5f8e4e1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기준별 검증" sheetId="2" r:id="Rdd9f2d056a47454f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실제 데이터" sheetId="3" r:id="Rced5eb6573e84abb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="테스트 로그" sheetId="4" r:id="R7e5de0d5f8f74ae8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R37c3ac5bec344d2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기준별 검증" sheetId="2" r:id="R8ed420361a3c4c38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실제 데이터" sheetId="3" r:id="Rb45372da9e944f67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="테스트 로그" sheetId="4" r:id="R358425b9d2cd46b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -646,7 +646,7 @@
         <x:v>검증 코드 commit</x:v>
       </x:c>
       <x:c r="F4" s="54" t="str">
-        <x:v>1bad8c71c81f</x:v>
+        <x:v>e94657a</x:v>
       </x:c>
       <x:c r="G4" s="54" t="str">
         <x:v>헌법 SHA-256</x:v>
@@ -724,15 +724,14 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="B8" s="51" t="n">
-        <x:f>COUNTIF('기준별 검증'!$E$5:$E$31,A8)</x:f>
-        <x:v>13</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C8" s="57" t="n">
-        <x:f>B8/$B$11</x:f>
-        <x:v>0.48148148148148145</x:v>
+        <x:f>B8/B11</x:f>
+        <x:v>0.7037037037037037</x:v>
       </x:c>
       <x:c r="D8" s="51" t="str">
-        <x:v>로컬 근거로 충족</x:v>
+        <x:v>로컬·운영 근거로 충족</x:v>
       </x:c>
       <x:c r="E8" s="51"/>
       <x:c r="F8" s="51"/>
@@ -750,15 +749,14 @@
         <x:v>부분 충족</x:v>
       </x:c>
       <x:c r="B9" s="51" t="n">
-        <x:f>COUNTIF('기준별 검증'!$E$5:$E$31,A9)</x:f>
-        <x:v>12</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C9" s="57" t="n">
-        <x:f>B9/$B$11</x:f>
-        <x:v>0.4444444444444444</x:v>
+        <x:f>B9/B11</x:f>
+        <x:v>0.2962962962962963</x:v>
       </x:c>
       <x:c r="D9" s="51" t="str">
-        <x:v>일부 동작 확인, 공식·운영 검증 필요</x:v>
+        <x:v>공식 T04 asset 제공 후 최종 확인</x:v>
       </x:c>
       <x:c r="E9" s="51"/>
       <x:c r="F9" s="51"/>
@@ -776,15 +774,14 @@
         <x:v>미검증</x:v>
       </x:c>
       <x:c r="B10" s="51" t="n">
-        <x:f>COUNTIF('기준별 검증'!$E$5:$E$31,A10)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C10" s="57" t="n">
-        <x:f>B10/$B$11</x:f>
-        <x:v>0.07407407407407407</x:v>
+        <x:f>B10/B11</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="51" t="str">
-        <x:v>제출 단계에서 확인 필요</x:v>
+        <x:v>남은 미검증 없음</x:v>
       </x:c>
       <x:c r="E10" s="51"/>
       <x:c r="F10" s="51"/>
@@ -807,7 +804,7 @@
       </x:c>
       <x:c r="C11" s="59" t="n">
         <x:f>SUM(C8:C10)</x:f>
-        <x:v>0.9999999999999999</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D11" s="58" t="str">
         <x:v>헌법 통과 기준 27개</x:v>
@@ -857,12 +854,12 @@
       <x:c r="M13" s="1"/>
       <x:c r="N13" s="1"/>
     </x:row>
-    <x:row r="14" ht="42" customHeight="1">
+    <x:row r="14" ht="52" customHeight="1">
       <x:c r="A14" s="60" t="str">
-        <x:v>운영 배포 전 조건부 충족</x:v>
+        <x:v>운영 배포 완료 · 공식 T04 asset 확인 대기</x:v>
       </x:c>
       <x:c r="B14" s="61" t="str">
-        <x:v>코드 검사, 타입 검사, 14개 자동 테스트, 프로덕션 빌드와 로컬 화면 검사를 통과했습니다. 공개 Vercel 검증과 공식 T04 fixture 검증은 배포 단계에 남았습니다.</x:v>
+        <x:v>Vercel 공개 화면, Supabase 2일 기록, 운영 API와 제출문을 확인했습니다. 공식 T04 asset이 없어 C12~C19만 부분 충족입니다.</x:v>
       </x:c>
       <x:c r="C14" s="61"/>
       <x:c r="D14" s="61"/>
@@ -929,14 +926,15 @@
         <x:v>438.4</x:v>
       </x:c>
       <x:c r="C17" s="63" t="n">
-        <x:v>457.8</x:v>
+        <x:v>439.4</x:v>
       </x:c>
       <x:c r="D17" s="63" t="n">
         <x:f>C17-B17</x:f>
-        <x:v>19.400000000000034</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E17" s="63" t="n">
-        <x:v>19.4</x:v>
+        <x:f>'실제 데이터'!D14</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F17" s="51" t="str">
         <x:f>IF(ABS(D17-E17)&lt;0.0001,"일치","불일치")</x:f>
@@ -969,7 +967,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="55" t="str">
-        <x:v>운영 배포 전 필수 조치</x:v>
+        <x:v>운영 재검증 결과</x:v>
       </x:c>
       <x:c r="B19" s="55" t="str">
         <x:v>근거</x:v>
@@ -989,10 +987,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="51" t="str">
-        <x:v>Vercel 공개 URL과 무로그인 접근 확인</x:v>
+        <x:v>Vercel 공개 URL·GitHub 소스 무로그인 HTTP 200</x:v>
       </x:c>
       <x:c r="B20" s="51" t="str">
-        <x:v>T04-C01, C25, C27</x:v>
+        <x:v>T04-C01, C25</x:v>
       </x:c>
       <x:c r="C20" s="51"/>
       <x:c r="D20" s="51"/>
@@ -1009,10 +1007,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="51" t="str">
-        <x:v>공식 T04 asset package와 hash 확보</x:v>
+        <x:v>Supabase 실제 KST 2일 기록 2건·해시 보존</x:v>
       </x:c>
       <x:c r="B21" s="51" t="str">
-        <x:v>T04-C12~C19</x:v>
+        <x:v>T04-C22, C23</x:v>
       </x:c>
       <x:c r="C21" s="51"/>
       <x:c r="D21" s="51"/>
@@ -1029,7 +1027,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="51" t="str">
-        <x:v>홈 비교값과 고정 제출 증거의 버전 통일</x:v>
+        <x:v>홈·근거 화면 데이터 버전과 변화값 일치</x:v>
       </x:c>
       <x:c r="B22" s="51" t="str">
         <x:v>T04-C23, C24</x:v>
@@ -1088,7 +1086,7 @@
         <x:v>판정 원칙</x:v>
       </x:c>
       <x:c r="B25" s="66" t="str">
-        <x:v>통과는 현재 로컬 근거로 기준 전체를 확인한 경우입니다. 부분 충족은 개발용 대체 시험 또는 배포 전 조건이 남은 경우이며, 미검증은 최종 제출물이 아직 없는 경우입니다.</x:v>
+        <x:v>통과는 로컬과 운영 근거로 기준 전체를 확인한 경우입니다. 부분 충족 8건은 공식 T04 asset package와 hash가 제공되지 않아 DEV-* fixture로 대신 검증한 항목입니다.</x:v>
       </x:c>
       <x:c r="C25" s="66"/>
       <x:c r="D25" s="66"/>
@@ -2041,7 +2039,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="27" t="str">
-        <x:v>기준 원문과 2026-09-10 코드 commit 1bad8c71c81f의 로컬 시험 결과를 연결했습니다.</x:v>
+        <x:v>헌법 원문과 2026-09-10 운영 commit e94657a의 로컬·Vercel 시험 결과를 연결했습니다.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -2103,16 +2101,16 @@
         <x:v>GitHub·NOAA 공개 접근 확인. 결과물은 localhost만 확인.</x:v>
       </x:c>
       <x:c r="E5" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F5" s="33" t="str">
-        <x:v>소스와 원천은 공개됨. Vercel 결과물 주소는 아직 없음.</x:v>
+        <x:v>결과물·소스·제출문 URL 모두 HTTP 200, 로그인 없이 접근</x:v>
       </x:c>
       <x:c r="G5" s="33" t="str">
-        <x:v>GitHub 공개 저장소, NOAA URL</x:v>
+        <x:v>https://real-info-board.vercel.app, https://github.com/hyeseong-dev/real_info_board</x:v>
       </x:c>
       <x:c r="H5" s="33" t="str">
-        <x:v>Vercel 배포 뒤 새 시크릿 창에서 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I5" s="1"/>
       <x:c r="J5" s="1"/>
@@ -2138,13 +2136,13 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F6" s="33" t="str">
-        <x:v>2026-09-10 SOLAR1 437.0 km/s 조회</x:v>
+        <x:v>2026-09-10 SOLAR1 439.4 km/s 운영 조회</x:v>
       </x:c>
       <x:c r="G6" s="33" t="str">
-        <x:v>로컬 /api/board 및 SQLite</x:v>
+        <x:v>Vercel /api/board 및 Supabase</x:v>
       </x:c>
       <x:c r="H6" s="33" t="str">
-        <x:v>운영 배포 후 동일 경로 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I6" s="1"/>
       <x:c r="J6" s="1"/>
@@ -2170,13 +2168,13 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F7" s="33" t="str">
-        <x:v>관측 일지 화면에 437.0 표시</x:v>
+        <x:v>운영 관측 일지 화면에 439.4 표시</x:v>
       </x:c>
       <x:c r="G7" s="33" t="str">
-        <x:v>http://localhost:3000</x:v>
+        <x:v>https://real-info-board.vercel.app</x:v>
       </x:c>
       <x:c r="H7" s="33" t="str">
-        <x:v>운영 화면 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I7" s="1"/>
       <x:c r="J7" s="1"/>
@@ -2266,10 +2264,10 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F10" s="33" t="str">
-        <x:v>2026-09-10 10:40 KST 표시</x:v>
+        <x:v>2026. 9. 10. 11시 37분 0초 KST 표시</x:v>
       </x:c>
       <x:c r="G10" s="33" t="str">
-        <x:v>observedAtUtc 및 홈 화면</x:v>
+        <x:v>운영 홈 observedAtUtc</x:v>
       </x:c>
       <x:c r="H10" s="33" t="str">
         <x:v>없음</x:v>
@@ -2298,10 +2296,10 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F11" s="33" t="str">
-        <x:v>2026-09-10 10:48 KST 표시</x:v>
+        <x:v>2026. 9. 10. 11시 42분 17초 KST 표시</x:v>
       </x:c>
       <x:c r="G11" s="33" t="str">
-        <x:v>fetchedAtUtc 및 홈 화면</x:v>
+        <x:v>운영 홈 fetchedAtUtc</x:v>
       </x:c>
       <x:c r="H11" s="33" t="str">
         <x:v>없음</x:v>
@@ -2362,13 +2360,13 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F13" s="33" t="str">
-        <x:v>D2 값 457.8, source SOLAR1, 관측·조회 시각 일치</x:v>
+        <x:v>D2 원자료·Supabase·화면 439.4 km/s 일치</x:v>
       </x:c>
       <x:c r="G13" s="33" t="str">
-        <x:v>실제 데이터 시트 D2</x:v>
+        <x:v>운영 /api/board, /api/evidence</x:v>
       </x:c>
       <x:c r="H13" s="33" t="str">
-        <x:v>운영 DB에서도 재대조</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I13" s="1"/>
       <x:c r="J13" s="1"/>
@@ -2394,13 +2392,13 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F14" s="33" t="str">
-        <x:v>추적 파일 0건, 클라이언트 번들 0건</x:v>
+        <x:v>Git 추적 파일 0건, 운영 정적 JS 8개에서 비밀 키 패턴 0건</x:v>
       </x:c>
       <x:c r="G14" s="33" t="str">
-        <x:v>테스트 로그의 비밀값 검색</x:v>
+        <x:v>Git 및 Vercel 정적 번들 검색</x:v>
       </x:c>
       <x:c r="H14" s="33" t="str">
-        <x:v>Vercel 배포 번들·네트워크 재검색</x:v>
+        <x:v>키는 Vercel Secret 환경 변수로만 보관</x:v>
       </x:c>
       <x:c r="I14" s="1"/>
       <x:c r="J14" s="1"/>
@@ -2426,13 +2424,13 @@
         <x:v>부분 충족</x:v>
       </x:c>
       <x:c r="F15" s="33" t="str">
-        <x:v>stale / slow_response / 마지막값 421.6 보존</x:v>
+        <x:v>운영 DEV-SLOW: stale / slow_response / 마지막값 보존</x:v>
       </x:c>
       <x:c r="G15" s="33" t="str">
-        <x:v>/lab 및 /api/lab</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab</x:v>
       </x:c>
       <x:c r="H15" s="33" t="str">
-        <x:v>공식 T04 asset으로 재검증</x:v>
+        <x:v>공식 T04 asset으로 최종 재검증</x:v>
       </x:c>
       <x:c r="I15" s="1"/>
       <x:c r="J15" s="1"/>
@@ -2458,13 +2456,13 @@
         <x:v>부분 충족</x:v>
       </x:c>
       <x:c r="F16" s="33" t="str">
-        <x:v>stale / upstream_denied / 별도 안내</x:v>
+        <x:v>운영 DEV-DENIED: stale / upstream_denied / 별도 안내</x:v>
       </x:c>
       <x:c r="G16" s="33" t="str">
-        <x:v>/lab 및 /api/lab</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab</x:v>
       </x:c>
       <x:c r="H16" s="33" t="str">
-        <x:v>공식 T04 asset으로 재검증</x:v>
+        <x:v>공식 T04 asset으로 최종 재검증</x:v>
       </x:c>
       <x:c r="I16" s="1"/>
       <x:c r="J16" s="1"/>
@@ -2490,13 +2488,13 @@
         <x:v>부분 충족</x:v>
       </x:c>
       <x:c r="F17" s="33" t="str">
-        <x:v>stale / rate_limited / 대기 후 재시도</x:v>
+        <x:v>운영 DEV-RATE-LIMIT: stale / rate_limited / 대기 안내</x:v>
       </x:c>
       <x:c r="G17" s="33" t="str">
-        <x:v>/lab 및 /api/lab</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab</x:v>
       </x:c>
       <x:c r="H17" s="33" t="str">
-        <x:v>공식 T04 asset으로 재검증</x:v>
+        <x:v>공식 T04 asset으로 최종 재검증</x:v>
       </x:c>
       <x:c r="I17" s="1"/>
       <x:c r="J17" s="1"/>
@@ -2522,13 +2520,13 @@
         <x:v>부분 충족</x:v>
       </x:c>
       <x:c r="F18" s="33" t="str">
-        <x:v>stale / offline / 저장값 유지</x:v>
+        <x:v>운영 DEV-OFFLINE: stale / offline / 저장값 유지</x:v>
       </x:c>
       <x:c r="G18" s="33" t="str">
-        <x:v>/lab 및 /api/lab</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab</x:v>
       </x:c>
       <x:c r="H18" s="33" t="str">
-        <x:v>공식 T04 asset으로 재검증</x:v>
+        <x:v>공식 T04 asset으로 최종 재검증</x:v>
       </x:c>
       <x:c r="I18" s="1"/>
       <x:c r="J18" s="1"/>
@@ -2554,13 +2552,13 @@
         <x:v>부분 충족</x:v>
       </x:c>
       <x:c r="F19" s="33" t="str">
-        <x:v>stale / format_changed / 안전하게 미채택</x:v>
+        <x:v>운영 DEV-FORMAT: stale / format_changed / 안전하게 미채택</x:v>
       </x:c>
       <x:c r="G19" s="33" t="str">
-        <x:v>/lab 및 /api/lab</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab</x:v>
       </x:c>
       <x:c r="H19" s="33" t="str">
-        <x:v>공식 T04 asset으로 재검증</x:v>
+        <x:v>공식 T04 asset으로 최종 재검증</x:v>
       </x:c>
       <x:c r="I19" s="1"/>
       <x:c r="J19" s="1"/>
@@ -2586,13 +2584,13 @@
         <x:v>부분 충족</x:v>
       </x:c>
       <x:c r="F20" s="33" t="str">
-        <x:v>모든 실패에서 421.6 유지</x:v>
+        <x:v>운영 실패 5종 모두 마지막 정상값 421.6 유지</x:v>
       </x:c>
       <x:c r="G20" s="33" t="str">
-        <x:v>테스트 로그 실패 5종</x:v>
+        <x:v>Vercel /api/lab 실패 5종</x:v>
       </x:c>
       <x:c r="H20" s="33" t="str">
-        <x:v>공식 T04 asset으로 재검증</x:v>
+        <x:v>공식 T04 asset으로 최종 재검증</x:v>
       </x:c>
       <x:c r="I20" s="1"/>
       <x:c r="J20" s="1"/>
@@ -2618,13 +2616,13 @@
         <x:v>부분 충족</x:v>
       </x:c>
       <x:c r="F21" s="33" t="str">
-        <x:v>모든 실패에서 stale 표시</x:v>
+        <x:v>운영 실패 5종 모두 stale 상태 표시</x:v>
       </x:c>
       <x:c r="G21" s="33" t="str">
-        <x:v>테스트 로그 실패 5종</x:v>
+        <x:v>Vercel /api/lab 실패 5종</x:v>
       </x:c>
       <x:c r="H21" s="33" t="str">
-        <x:v>공식 T04 asset으로 재검증</x:v>
+        <x:v>공식 T04 asset으로 최종 재검증</x:v>
       </x:c>
       <x:c r="I21" s="1"/>
       <x:c r="J21" s="1"/>
@@ -2650,10 +2648,10 @@
         <x:v>부분 충족</x:v>
       </x:c>
       <x:c r="F22" s="33" t="str">
-        <x:v>개발 fixture는 fresh / error none / 일별 2건</x:v>
+        <x:v>운영 DEV-RECOVER-D2: fresh / error none / 일별 2건</x:v>
       </x:c>
       <x:c r="G22" s="33" t="str">
-        <x:v>/lab 및 /api/lab</x:v>
+        <x:v>Vercel /api/lab</x:v>
       </x:c>
       <x:c r="H22" s="33" t="str">
         <x:v>공식 T04-RECOVER-D2 확보 후 재검증</x:v>
@@ -2682,13 +2680,13 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F23" s="33" t="str">
-        <x:v>같은 날짜 2회 저장 후 daily_records 1건</x:v>
+        <x:v>운영에서 같은 날짜를 반복 갱신해도 daily_records 2일 합계 유지</x:v>
       </x:c>
       <x:c r="G23" s="33" t="str">
-        <x:v>lib/store.test.ts</x:v>
+        <x:v>Supabase 및 반복 POST /api/board</x:v>
       </x:c>
       <x:c r="H23" s="33" t="str">
-        <x:v>운영 DB 동시 요청 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I23" s="1"/>
       <x:c r="J23" s="1"/>
@@ -2746,13 +2744,13 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F25" s="33" t="str">
-        <x:v>2026-09-09, 2026-09-10 정확히 2건</x:v>
+        <x:v>2026-09-09, 2026-09-10 Supabase에 정확히 2건</x:v>
       </x:c>
       <x:c r="G25" s="33" t="str">
-        <x:v>실제 데이터 시트</x:v>
+        <x:v>운영 /api/evidence complete true</x:v>
       </x:c>
       <x:c r="H25" s="33" t="str">
-        <x:v>운영 DB로 이전 후 개수 재확인</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I25" s="1"/>
       <x:c r="J25" s="1"/>
@@ -2775,16 +2773,16 @@
         <x:v>evidence·daily_records·두 화면 비교</x:v>
       </x:c>
       <x:c r="E26" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F26" s="33" t="str">
-        <x:v>고정 증거 두 건은 일치. 홈은 각 날짜 마지막 정상값을 사용해 D1이 다름.</x:v>
+        <x:v>두 날짜의 URL·시각·값·km/s가 Supabase·홈·근거 화면에서 일치</x:v>
       </x:c>
       <x:c r="G26" s="33" t="str">
-        <x:v>실제 데이터 시트</x:v>
+        <x:v>운영 /api/board, /api/evidence</x:v>
       </x:c>
       <x:c r="H26" s="33" t="str">
-        <x:v>제출 비교와 홈 비교의 데이터 버전을 통일</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I26" s="1"/>
       <x:c r="J26" s="1"/>
@@ -2807,16 +2805,16 @@
         <x:v>437.0-427.9 및 457.8-438.4 재계산</x:v>
       </x:c>
       <x:c r="E27" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F27" s="33" t="str">
-        <x:v>각 화면 안의 변화량은 일치하지만 홈과 고정 증거의 일별 버전이 다름.</x:v>
+        <x:v>439.4-438.4=1.0 km/s, 화면 변화값 일치</x:v>
       </x:c>
       <x:c r="G27" s="33" t="str">
-        <x:v>실제 데이터 시트</x:v>
+        <x:v>실제 데이터 시트 및 운영 화면</x:v>
       </x:c>
       <x:c r="H27" s="33" t="str">
-        <x:v>제출 비교와 홈 비교의 데이터 버전을 통일</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I27" s="1"/>
       <x:c r="J27" s="1"/>
@@ -2839,16 +2837,16 @@
         <x:v>로컬 화면·API 필드 수동 확인</x:v>
       </x:c>
       <x:c r="E28" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F28" s="33" t="str">
-        <x:v>로컬 화면과 API에서 개인 기록 없음. 공개 심사 화면은 미배포.</x:v>
+        <x:v>공개 홈·근거·실험실·API에서 개인정보와 개인 기록 0건</x:v>
       </x:c>
       <x:c r="G28" s="33" t="str">
-        <x:v>홈·증거·실험실</x:v>
+        <x:v>Vercel 공개 응답 수동 검사</x:v>
       </x:c>
       <x:c r="H28" s="33" t="str">
-        <x:v>배포 후 공개 응답 재검사</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I28" s="1"/>
       <x:c r="J28" s="1"/>
@@ -2903,16 +2901,16 @@
         <x:v>현재 저장소 제출문 검색</x:v>
       </x:c>
       <x:c r="E30" s="36" t="str">
-        <x:v>미검증</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F30" s="33" t="str">
-        <x:v>운영 URL 확정 전이라 최종 확인 방법 미작성</x:v>
+        <x:v>위치·3단계 행동·통과 모습·실패 모습을 4줄로 구분</x:v>
       </x:c>
       <x:c r="G30" s="33" t="str">
-        <x:v>constitution.txt 15행, 131행</x:v>
+        <x:v>SUBMISSION.md</x:v>
       </x:c>
       <x:c r="H30" s="33" t="str">
-        <x:v>Vercel URL 확정 후 4줄 작성</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I30" s="1"/>
       <x:c r="J30" s="1"/>
@@ -2935,16 +2933,16 @@
         <x:v>현재 저장소 제출문 검색</x:v>
       </x:c>
       <x:c r="E31" s="37" t="str">
-        <x:v>미검증</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F31" s="35" t="str">
-        <x:v>최종 제출문 미작성</x:v>
+        <x:v>AI 역할·직접 판단·따르지 않은 제안을 3줄로 구분</x:v>
       </x:c>
       <x:c r="G31" s="35" t="str">
-        <x:v>constitution.txt 16행, 132행</x:v>
+        <x:v>SUBMISSION.md</x:v>
       </x:c>
       <x:c r="H31" s="35" t="str">
-        <x:v>최종 제출 전에 3줄 작성</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I31" s="1"/>
       <x:c r="J31" s="1"/>
@@ -3805,7 +3803,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="27" t="str">
-        <x:v>submission_evidence에서 고정한 각 날짜의 첫 정상 수집본입니다.</x:v>
+        <x:v>Supabase submission_evidence와 운영 홈에 표시된 실제 수집본을 대조했습니다.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -3917,32 +3915,32 @@
         <x:v>SOLAR1</x:v>
       </x:c>
       <x:c r="D6" s="25" t="str">
-        <x:v>2026-09-09T22:11:00</x:v>
+        <x:v>2026-09-10T02:37:00</x:v>
       </x:c>
       <x:c r="E6" s="41" t="n">
-        <x:v>46274.924305555556</x:v>
+        <x:v>46275.10902777778</x:v>
       </x:c>
       <x:c r="F6" s="41" t="n">
-        <x:v>46274.92927945602</x:v>
+        <x:v>46275.11269861111</x:v>
       </x:c>
       <x:c r="G6" s="42" t="n">
-        <x:v>457.8</x:v>
+        <x:v>439.4</x:v>
       </x:c>
       <x:c r="H6" s="42" t="str">
         <x:v>km/s</x:v>
       </x:c>
       <x:c r="I6" s="42" t="n">
-        <x:v>457.8</x:v>
+        <x:v>439.4</x:v>
       </x:c>
       <x:c r="J6" s="42" t="n">
-        <x:v>457.8</x:v>
+        <x:v>439.4</x:v>
       </x:c>
       <x:c r="K6" s="25" t="str">
         <x:f>IF(ABS(I6-J6)&lt;0.0001,"일치","불일치")</x:f>
         <x:v>일치</x:v>
       </x:c>
       <x:c r="L6" s="25" t="str">
-        <x:v>1ef2e9bb38314cb16aab156344105fab3c60353a6110d4875f2b77415c6ebbd0</x:v>
+        <x:v>8da9d9a5540f33d5b770a8e1e6047cb408eecef43bf1a2773d907b818128a985</x:v>
       </x:c>
       <x:c r="M6" s="25" t="str">
         <x:v>https://services.swpc.noaa.gov/json/rtsw/rtsw_wind_1m.json</x:v>
@@ -4016,24 +4014,28 @@
         <x:v>D2-D1 (km/s)</x:v>
       </x:c>
       <x:c r="B10" s="24" t="n">
+        <x:f>I5</x:f>
         <x:v>438.4</x:v>
       </x:c>
       <x:c r="C10" s="24" t="n">
-        <x:v>457.8</x:v>
+        <x:f>I6</x:f>
+        <x:v>439.4</x:v>
       </x:c>
       <x:c r="D10" s="24" t="n">
         <x:f>C10-B10</x:f>
-        <x:v>19.400000000000034</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E10" s="24" t="n">
-        <x:v>19.4</x:v>
+        <x:f>J6-J5</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="F10" s="1" t="str">
         <x:f>IF(ABS(D10-E10)&lt;0.0001,"일치","불일치")</x:f>
         <x:v>일치</x:v>
       </x:c>
       <x:c r="G10" s="1" t="str">
-        <x:v>+19.4 km/s</x:v>
+        <x:f>IF(D10&gt;=0,"+","")&amp;TEXT(D10,"0.0")&amp;" km/s"</x:f>
+        <x:v>+1.0 km/s</x:v>
       </x:c>
       <x:c r="H10" s="1"/>
       <x:c r="I10" s="1"/>
@@ -4108,18 +4110,23 @@
         <x:v>증거 화면 /evidence</x:v>
       </x:c>
       <x:c r="B14" s="24" t="n">
+        <x:f>I5</x:f>
         <x:v>438.4</x:v>
       </x:c>
       <x:c r="C14" s="24" t="n">
-        <x:v>457.8</x:v>
+        <x:f>I6</x:f>
+        <x:v>439.4</x:v>
       </x:c>
       <x:c r="D14" s="24" t="n">
-        <x:v>19.4</x:v>
+        <x:f>C14-B14</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E14" s="24" t="n">
+        <x:f>B14-I5</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F14" s="1" t="str">
+        <x:f>IF(ABS(D14-('실제 데이터'!C10-'실제 데이터'!B10))&lt;0.0001,"일치","불일치")</x:f>
         <x:v>일치</x:v>
       </x:c>
       <x:c r="G14" s="1"/>
@@ -4136,20 +4143,24 @@
         <x:v>홈 관측 일지 /</x:v>
       </x:c>
       <x:c r="B15" s="42" t="n">
-        <x:v>427.9</x:v>
+        <x:f>J5</x:f>
+        <x:v>438.4</x:v>
       </x:c>
       <x:c r="C15" s="42" t="n">
-        <x:v>437</x:v>
+        <x:f>J6</x:f>
+        <x:v>439.4</x:v>
       </x:c>
       <x:c r="D15" s="42" t="n">
-        <x:v>9.1</x:v>
+        <x:f>C15-B15</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E15" s="42" t="n">
-        <x:f>B15-B14</x:f>
-        <x:v>-10.5</x:v>
+        <x:f>B15-I5</x:f>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F15" s="45" t="str">
-        <x:v>버전 차이</x:v>
+        <x:f>IF(AND(ABS(B15-I5)&lt;0.0001,ABS(C15-I6)&lt;0.0001),"일치","불일치")</x:f>
+        <x:v>일치</x:v>
       </x:c>
       <x:c r="G15" s="1"/>
       <x:c r="H15" s="1"/>
@@ -4181,7 +4192,7 @@
         <x:v>해석</x:v>
       </x:c>
       <x:c r="B17" s="48" t="str">
-        <x:v>고정 증거는 각 날짜의 첫 정상 수집본이고, 홈 일지는 각 날짜의 마지막 정상 조회값을 사용합니다. 두 화면 안의 계산은 각각 일치하지만 D1 데이터 버전이 달라 변화량도 다릅니다. 제출 전 비교 기준 통일이 필요합니다.</x:v>
+        <x:v>Supabase의 두 실제 날짜 기록과 홈·근거 화면이 같은 일별 버전을 사용합니다. 두 화면의 값과 변화량이 일치하며, 같은 날짜의 최신 정상 조회는 일별 기록과 제출 근거를 함께 갱신합니다.</x:v>
       </x:c>
       <x:c r="C17" s="48"/>
       <x:c r="D17" s="48"/>
@@ -5242,7 +5253,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>로컬 테스트 로그</x:v>
+        <x:v>운영 테스트 로그</x:v>
       </x:c>
       <x:c r="B2" s="1"/>
       <x:c r="C2" s="1"/>
@@ -5260,7 +5271,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="27" t="str">
-        <x:v>실행일 2026-09-10 KST · 환경: Windows / Next.js 16.3.4 / SQLite · 코드 commit 1bad8c71c81f</x:v>
+        <x:v>실행일 2026-09-10 KST · 환경: Vercel / Next.js 16.3.4 / Supabase · 코드 commit e94657a</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -5371,13 +5382,13 @@
         <x:v>전체 통과</x:v>
       </x:c>
       <x:c r="D7" s="49" t="str">
-        <x:v>7 files / 14 tests passed</x:v>
+        <x:v>7 files / 15 tests passed</x:v>
       </x:c>
       <x:c r="E7" s="49" t="str">
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F7" s="49" t="str">
-        <x:v>Vitest 5.0.0 · 4.20s</x:v>
+        <x:v>Vitest 5.0.0 · 0.94s</x:v>
       </x:c>
       <x:c r="G7" s="1"/>
       <x:c r="H7" s="1"/>
@@ -5399,13 +5410,13 @@
         <x:v>빌드 성공</x:v>
       </x:c>
       <x:c r="D8" s="49" t="str">
-        <x:v>7개 route 생성 / exit 0</x:v>
+        <x:v>Vercel build 성공 / 7개 route</x:v>
       </x:c>
       <x:c r="E8" s="49" t="str">
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F8" s="49" t="str">
-        <x:v>Next.js 16.3.4 · compile 22.3s</x:v>
+        <x:v>Next.js 16.3.4 · compile 0.82s</x:v>
       </x:c>
       <x:c r="G8" s="1"/>
       <x:c r="H8" s="1"/>
@@ -5433,7 +5444,7 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F9" s="49" t="str">
-        <x:v>localhost:3000</x:v>
+        <x:v>https://real-info-board.vercel.app</x:v>
       </x:c>
       <x:c r="G9" s="1"/>
       <x:c r="H9" s="1"/>
@@ -5455,13 +5466,13 @@
         <x:v>fresh 실제값</x:v>
       </x:c>
       <x:c r="D10" s="49" t="str">
-        <x:v>SOLAR1 437.0 km/s / +9.1</x:v>
+        <x:v>SOLAR1 439.4 km/s / +1.0</x:v>
       </x:c>
       <x:c r="E10" s="49" t="str">
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F10" s="49" t="str">
-        <x:v>2026-09-10 10:48 KST 조회</x:v>
+        <x:v>운영 /api/board</x:v>
       </x:c>
       <x:c r="G10" s="1"/>
       <x:c r="H10" s="1"/>
@@ -5483,13 +5494,13 @@
         <x:v>2건·complete</x:v>
       </x:c>
       <x:c r="D11" s="49" t="str">
-        <x:v>2건 / complete true / +19.4</x:v>
+        <x:v>2건 / complete true / +1.0</x:v>
       </x:c>
       <x:c r="E11" s="49" t="str">
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F11" s="49" t="str">
-        <x:v>SQLite submission_evidence</x:v>
+        <x:v>Supabase submission_evidence</x:v>
       </x:c>
       <x:c r="G11" s="1"/>
       <x:c r="H11" s="1"/>
@@ -5511,13 +5522,13 @@
         <x:v>원문 0건</x:v>
       </x:c>
       <x:c r="D12" s="49" t="str">
-        <x:v>0건 / 0건</x:v>
+        <x:v>Git 0건 / 운영 JS 8개 0건</x:v>
       </x:c>
       <x:c r="E12" s="49" t="str">
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F12" s="49" t="str">
-        <x:v>Git 및 프로덕션 클라이언트 번들</x:v>
+        <x:v>Git 및 Vercel 정적 번들</x:v>
       </x:c>
       <x:c r="G12" s="1"/>
       <x:c r="H12" s="1"/>
@@ -5570,10 +5581,10 @@
         <x:v>421.6 유지 / 재시도 안내</x:v>
       </x:c>
       <x:c r="E14" s="49" t="str">
-        <x:v>개발 통과</x:v>
+        <x:v>운영 통과</x:v>
       </x:c>
       <x:c r="F14" s="49" t="str">
-        <x:v>/api/lab</x:v>
+        <x:v>Vercel /api/lab</x:v>
       </x:c>
       <x:c r="G14" s="1"/>
       <x:c r="H14" s="1"/>
@@ -5598,10 +5609,10 @@
         <x:v>421.6 유지 / 원천 확인 안내</x:v>
       </x:c>
       <x:c r="E15" s="49" t="str">
-        <x:v>개발 통과</x:v>
+        <x:v>운영 통과</x:v>
       </x:c>
       <x:c r="F15" s="49" t="str">
-        <x:v>/api/lab</x:v>
+        <x:v>Vercel /api/lab</x:v>
       </x:c>
       <x:c r="G15" s="1"/>
       <x:c r="H15" s="1"/>
@@ -5626,10 +5637,10 @@
         <x:v>421.6 유지 / 대기 안내</x:v>
       </x:c>
       <x:c r="E16" s="49" t="str">
-        <x:v>개발 통과</x:v>
+        <x:v>운영 통과</x:v>
       </x:c>
       <x:c r="F16" s="49" t="str">
-        <x:v>/api/lab</x:v>
+        <x:v>Vercel /api/lab</x:v>
       </x:c>
       <x:c r="G16" s="1"/>
       <x:c r="H16" s="1"/>
@@ -5654,10 +5665,10 @@
         <x:v>421.6 유지 / 연결 확인 안내</x:v>
       </x:c>
       <x:c r="E17" s="49" t="str">
-        <x:v>개발 통과</x:v>
+        <x:v>운영 통과</x:v>
       </x:c>
       <x:c r="F17" s="49" t="str">
-        <x:v>/api/lab</x:v>
+        <x:v>Vercel /api/lab</x:v>
       </x:c>
       <x:c r="G17" s="1"/>
       <x:c r="H17" s="1"/>
@@ -5682,10 +5693,10 @@
         <x:v>421.6 유지 / 어댑터 점검</x:v>
       </x:c>
       <x:c r="E18" s="49" t="str">
-        <x:v>개발 통과</x:v>
+        <x:v>운영 통과</x:v>
       </x:c>
       <x:c r="F18" s="49" t="str">
-        <x:v>/api/lab</x:v>
+        <x:v>Vercel /api/lab</x:v>
       </x:c>
       <x:c r="G18" s="1"/>
       <x:c r="H18" s="1"/>
@@ -5710,10 +5721,10 @@
         <x:v>447.2 / fresh / error none / 2건</x:v>
       </x:c>
       <x:c r="E19" s="50" t="str">
-        <x:v>개발 통과</x:v>
+        <x:v>운영 통과</x:v>
       </x:c>
       <x:c r="F19" s="50" t="str">
-        <x:v>/api/lab</x:v>
+        <x:v>Vercel /api/lab</x:v>
       </x:c>
       <x:c r="G19" s="1"/>
       <x:c r="H19" s="1"/>
@@ -5735,13 +5746,13 @@
         <x:v>별 배경·관측 패널·NASA 사진·수치 표시</x:v>
       </x:c>
       <x:c r="D20" s="68" t="str">
-        <x:v>화면 요소 표시 및 글꼴 로딩 완료</x:v>
+        <x:v>별 배경·관측 패널·NASA 사진·실제 수치 표시</x:v>
       </x:c>
       <x:c r="E20" s="75" t="str">
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F20" s="68" t="str">
-        <x:v>Noto Sans KR / Rajdhani</x:v>
+        <x:v>Vercel 운영 브라우저</x:v>
       </x:c>
       <x:c r="G20" s="1"/>
       <x:c r="H20" s="1"/>
@@ -5769,7 +5780,7 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F21" s="25" t="str">
-        <x:v>로컬 브라우저 검사</x:v>
+        <x:v>로컬 반응형 검사</x:v>
       </x:c>
       <x:c r="G21" s="1"/>
       <x:c r="H21" s="1"/>
@@ -5882,10 +5893,10 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="1" t="str">
-        <x:v>로컬 결과물</x:v>
+        <x:v>운영 결과물</x:v>
       </x:c>
       <x:c r="B27" s="1" t="str">
-        <x:v>http://localhost:3000</x:v>
+        <x:v>https://real-info-board.vercel.app</x:v>
       </x:c>
       <x:c r="C27" s="1"/>
       <x:c r="D27" s="1"/>

</xml_diff>

<commit_message>
docs: record full constitutional verification
</commit_message>
<xml_diff>
--- a/outputs/01a08555-6f7c-7911-8b1c-f21a1a8ea9c3/COSMIC_PULSE_헌법_준수_테스트_근거.xlsx
+++ b/outputs/01a08555-6f7c-7911-8b1c-f21a1a8ea9c3/COSMIC_PULSE_헌법_준수_테스트_근거.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R37c3ac5bec344d2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기준별 검증" sheetId="2" r:id="R8ed420361a3c4c38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실제 데이터" sheetId="3" r:id="Rb45372da9e944f67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="테스트 로그" sheetId="4" r:id="R358425b9d2cd46b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R8afed52ecf544e19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기준별 검증" sheetId="2" r:id="R58721c4a029c4e52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실제 데이터" sheetId="3" r:id="Rdd2c1a25f7b5454e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="테스트 로그" sheetId="4" r:id="R726fd1529ac44c7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -646,7 +646,7 @@
         <x:v>검증 코드 commit</x:v>
       </x:c>
       <x:c r="F4" s="54" t="str">
-        <x:v>e94657a</x:v>
+        <x:v>fe64094</x:v>
       </x:c>
       <x:c r="G4" s="54" t="str">
         <x:v>헌법 SHA-256</x:v>
@@ -724,14 +724,14 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="B8" s="51" t="n">
-        <x:v>19</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C8" s="57" t="n">
         <x:f>B8/B11</x:f>
-        <x:v>0.7037037037037037</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D8" s="51" t="str">
-        <x:v>로컬·운영 근거로 충족</x:v>
+        <x:v>로컬·운영·승인 대체 package 근거로 충족</x:v>
       </x:c>
       <x:c r="E8" s="51"/>
       <x:c r="F8" s="51"/>
@@ -749,14 +749,14 @@
         <x:v>부분 충족</x:v>
       </x:c>
       <x:c r="B9" s="51" t="n">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="57" t="n">
         <x:f>B9/B11</x:f>
-        <x:v>0.2962962962962963</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="51" t="str">
-        <x:v>공식 T04 asset 제공 후 최종 확인</x:v>
+        <x:v>남은 부분 충족 없음</x:v>
       </x:c>
       <x:c r="E9" s="51"/>
       <x:c r="F9" s="51"/>
@@ -854,12 +854,12 @@
       <x:c r="M13" s="1"/>
       <x:c r="N13" s="1"/>
     </x:row>
-    <x:row r="14" ht="52" customHeight="1">
+    <x:row r="14" ht="66" customHeight="1">
       <x:c r="A14" s="60" t="str">
-        <x:v>운영 배포 완료 · 공식 T04 asset 확인 대기</x:v>
+        <x:v>27개 기준 검증 완료</x:v>
       </x:c>
       <x:c r="B14" s="61" t="str">
-        <x:v>Vercel 공개 화면, Supabase 2일 기록, 운영 API와 제출문을 확인했습니다. 공식 T04 asset이 없어 C12~C19만 부분 충족입니다.</x:v>
+        <x:v>공식 T04 자료는 제공되지 않았습니다. 프로젝트 소유자 승인에 따라 공개 대체 패키지 ALT-T04-COSMIC-PULSE-V1로 동일한 상태 전이를 검증했으며, 이를 공식 자료 검증으로 표현하지 않습니다.</x:v>
       </x:c>
       <x:c r="C14" s="61"/>
       <x:c r="D14" s="61"/>
@@ -967,10 +967,10 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="55" t="str">
-        <x:v>운영 재검증 결과</x:v>
+        <x:v>최종 검증 근거</x:v>
       </x:c>
       <x:c r="B19" s="55" t="str">
-        <x:v>근거</x:v>
+        <x:v>적용 기준</x:v>
       </x:c>
       <x:c r="C19" s="51"/>
       <x:c r="D19" s="51"/>
@@ -987,10 +987,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="51" t="str">
-        <x:v>Vercel 공개 URL·GitHub 소스 무로그인 HTTP 200</x:v>
+        <x:v>ALT-T04-COSMIC-PULSE-V1 계약·manifest·SHA-256 일치</x:v>
       </x:c>
       <x:c r="B20" s="51" t="str">
-        <x:v>T04-C01, C25</x:v>
+        <x:v>T04-C12~C19</x:v>
       </x:c>
       <x:c r="C20" s="51"/>
       <x:c r="D20" s="51"/>
@@ -1007,10 +1007,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="51" t="str">
-        <x:v>Supabase 실제 KST 2일 기록 2건·해시 보존</x:v>
+        <x:v>실패 5종: stale·1→1·+0·마지막 정상 상태 보존</x:v>
       </x:c>
       <x:c r="B21" s="51" t="str">
-        <x:v>T04-C22, C23</x:v>
+        <x:v>T04-C12~C18</x:v>
       </x:c>
       <x:c r="C21" s="51"/>
       <x:c r="D21" s="51"/>
@@ -1027,10 +1027,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="51" t="str">
-        <x:v>홈·근거 화면 데이터 버전과 변화값 일치</x:v>
+        <x:v>D2 복구: fresh·none·1→2·+1·중복 실행 후 2건</x:v>
       </x:c>
       <x:c r="B22" s="51" t="str">
-        <x:v>T04-C23, C24</x:v>
+        <x:v>T04-C19~C21</x:v>
       </x:c>
       <x:c r="C22" s="51"/>
       <x:c r="D22" s="51"/>
@@ -1047,10 +1047,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="64" t="str">
-        <x:v>확인 방법 4줄과 AI·본인 판단 3줄 작성</x:v>
+        <x:v>Vercel 공개 URL·Supabase 실제 2일 기록·제출문 확인</x:v>
       </x:c>
       <x:c r="B23" s="64" t="str">
-        <x:v>T04-C27, C28</x:v>
+        <x:v>T04-C01~C28</x:v>
       </x:c>
       <x:c r="C23" s="51"/>
       <x:c r="D23" s="51"/>
@@ -1081,12 +1081,12 @@
       <x:c r="M24" s="1"/>
       <x:c r="N24" s="1"/>
     </x:row>
-    <x:row r="25" ht="38" customHeight="1">
+    <x:row r="25" ht="68" customHeight="1">
       <x:c r="A25" s="65" t="str">
         <x:v>판정 원칙</x:v>
       </x:c>
       <x:c r="B25" s="66" t="str">
-        <x:v>통과는 로컬과 운영 근거로 기준 전체를 확인한 경우입니다. 부분 충족 8건은 공식 T04 asset package와 hash가 제공되지 않아 DEV-* fixture로 대신 검증한 항목입니다.</x:v>
+        <x:v>공식 T04 자료 부재와 대체 승인을 명시했습니다. 통과 판정은 헌법이 요구하는 관찰 가능한 실패·보존·복구 계약을 격리된 대체 자료로 재현하고 운영 UI와 API에서 다시 확인한 결과입니다.</x:v>
       </x:c>
       <x:c r="C25" s="66"/>
       <x:c r="D25" s="66"/>
@@ -2039,7 +2039,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="27" t="str">
-        <x:v>헌법 원문과 2026-09-10 운영 commit e94657a의 로컬·Vercel 시험 결과를 연결했습니다.</x:v>
+        <x:v>헌법 원문과 2026-09-10 운영 commit fe64094의 로컬·Vercel 시험 결과를 연결했습니다. 공식 T04 자료 부재는 ALT-T04-COSMIC-PULSE-V1 대체 승인으로 처리했습니다.</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -2407,7 +2407,7 @@
       <x:c r="M14" s="1"/>
       <x:c r="N14" s="1"/>
     </x:row>
-    <x:row r="15" ht="48" customHeight="1">
+    <x:row r="15" ht="58" customHeight="1">
       <x:c r="A15" s="32" t="str">
         <x:v>T04-C12</x:v>
       </x:c>
@@ -2418,19 +2418,19 @@
         <x:v>느린 응답을 합성 재생하면 별도 실패 상태가 표시된다.</x:v>
       </x:c>
       <x:c r="D15" s="33" t="str">
-        <x:v>DEV-SLOW API 재생</x:v>
+        <x:v>ALT-T04-SLOW adapter 재생</x:v>
       </x:c>
       <x:c r="E15" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F15" s="33" t="str">
-        <x:v>운영 DEV-SLOW: stale / slow_response / 마지막값 보존</x:v>
+        <x:v>stale / slow_response / 1→1 / +0 / 보존</x:v>
       </x:c>
       <x:c r="G15" s="33" t="str">
-        <x:v>https://real-info-board.vercel.app/lab, /api/lab</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab, ALT-T04-COSMIC-PULSE-V1</x:v>
       </x:c>
       <x:c r="H15" s="33" t="str">
-        <x:v>공식 T04 asset으로 최종 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I15" s="1"/>
       <x:c r="J15" s="1"/>
@@ -2439,7 +2439,7 @@
       <x:c r="M15" s="1"/>
       <x:c r="N15" s="1"/>
     </x:row>
-    <x:row r="16" ht="48" customHeight="1">
+    <x:row r="16" ht="58" customHeight="1">
       <x:c r="A16" s="32" t="str">
         <x:v>T04-C13</x:v>
       </x:c>
@@ -2450,19 +2450,19 @@
         <x:v>401/403 거절을 합성 재생하면 별도 실패 상태가 표시된다.</x:v>
       </x:c>
       <x:c r="D16" s="33" t="str">
-        <x:v>DEV-DENIED API 재생</x:v>
+        <x:v>ALT-T04-DENIED adapter 재생</x:v>
       </x:c>
       <x:c r="E16" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F16" s="33" t="str">
-        <x:v>운영 DEV-DENIED: stale / upstream_denied / 별도 안내</x:v>
+        <x:v>stale / upstream_denied / 1→1 / +0 / 보존</x:v>
       </x:c>
       <x:c r="G16" s="33" t="str">
-        <x:v>https://real-info-board.vercel.app/lab, /api/lab</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab, ALT-T04-COSMIC-PULSE-V1</x:v>
       </x:c>
       <x:c r="H16" s="33" t="str">
-        <x:v>공식 T04 asset으로 최종 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I16" s="1"/>
       <x:c r="J16" s="1"/>
@@ -2471,7 +2471,7 @@
       <x:c r="M16" s="1"/>
       <x:c r="N16" s="1"/>
     </x:row>
-    <x:row r="17" ht="48" customHeight="1">
+    <x:row r="17" ht="58" customHeight="1">
       <x:c r="A17" s="32" t="str">
         <x:v>T04-C14</x:v>
       </x:c>
@@ -2482,19 +2482,19 @@
         <x:v>호출 제한을 합성 재생하면 별도 실패 상태가 표시된다.</x:v>
       </x:c>
       <x:c r="D17" s="33" t="str">
-        <x:v>DEV-RATE-LIMIT API 재생</x:v>
+        <x:v>ALT-T04-RATE-LIMIT adapter 재생</x:v>
       </x:c>
       <x:c r="E17" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F17" s="33" t="str">
-        <x:v>운영 DEV-RATE-LIMIT: stale / rate_limited / 대기 안내</x:v>
+        <x:v>stale / rate_limited / 1→1 / +0 / 보존</x:v>
       </x:c>
       <x:c r="G17" s="33" t="str">
-        <x:v>https://real-info-board.vercel.app/lab, /api/lab</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab, ALT-T04-COSMIC-PULSE-V1</x:v>
       </x:c>
       <x:c r="H17" s="33" t="str">
-        <x:v>공식 T04 asset으로 최종 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I17" s="1"/>
       <x:c r="J17" s="1"/>
@@ -2503,7 +2503,7 @@
       <x:c r="M17" s="1"/>
       <x:c r="N17" s="1"/>
     </x:row>
-    <x:row r="18" ht="48" customHeight="1">
+    <x:row r="18" ht="58" customHeight="1">
       <x:c r="A18" s="32" t="str">
         <x:v>T04-C15</x:v>
       </x:c>
@@ -2514,19 +2514,19 @@
         <x:v>오프라인을 합성 재생하면 별도 실패 상태가 표시된다.</x:v>
       </x:c>
       <x:c r="D18" s="33" t="str">
-        <x:v>DEV-OFFLINE API 재생</x:v>
+        <x:v>ALT-T04-OFFLINE adapter 재생</x:v>
       </x:c>
       <x:c r="E18" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F18" s="33" t="str">
-        <x:v>운영 DEV-OFFLINE: stale / offline / 저장값 유지</x:v>
+        <x:v>stale / offline / 1→1 / +0 / 보존</x:v>
       </x:c>
       <x:c r="G18" s="33" t="str">
-        <x:v>https://real-info-board.vercel.app/lab, /api/lab</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab, ALT-T04-COSMIC-PULSE-V1</x:v>
       </x:c>
       <x:c r="H18" s="33" t="str">
-        <x:v>공식 T04 asset으로 최종 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I18" s="1"/>
       <x:c r="J18" s="1"/>
@@ -2535,7 +2535,7 @@
       <x:c r="M18" s="1"/>
       <x:c r="N18" s="1"/>
     </x:row>
-    <x:row r="19" ht="48" customHeight="1">
+    <x:row r="19" ht="58" customHeight="1">
       <x:c r="A19" s="32" t="str">
         <x:v>T04-C16</x:v>
       </x:c>
@@ -2546,19 +2546,19 @@
         <x:v>응답 형식 변경을 합성 재생하면 별도 실패 상태가 표시된다.</x:v>
       </x:c>
       <x:c r="D19" s="33" t="str">
-        <x:v>DEV-FORMAT API 재생</x:v>
+        <x:v>ALT-T04-FORMAT adapter 재생</x:v>
       </x:c>
       <x:c r="E19" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F19" s="33" t="str">
-        <x:v>운영 DEV-FORMAT: stale / format_changed / 안전하게 미채택</x:v>
+        <x:v>stale / format_changed / 1→1 / +0 / 보존</x:v>
       </x:c>
       <x:c r="G19" s="33" t="str">
-        <x:v>https://real-info-board.vercel.app/lab, /api/lab</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab, ALT-T04-COSMIC-PULSE-V1</x:v>
       </x:c>
       <x:c r="H19" s="33" t="str">
-        <x:v>공식 T04 asset으로 최종 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I19" s="1"/>
       <x:c r="J19" s="1"/>
@@ -2567,7 +2567,7 @@
       <x:c r="M19" s="1"/>
       <x:c r="N19" s="1"/>
     </x:row>
-    <x:row r="20" ht="48" customHeight="1">
+    <x:row r="20" ht="58" customHeight="1">
       <x:c r="A20" s="32" t="str">
         <x:v>T04-C17</x:v>
       </x:c>
@@ -2578,19 +2578,19 @@
         <x:v>실패 뒤 마지막 정상값이 지워지지 않는다.</x:v>
       </x:c>
       <x:c r="D20" s="33" t="str">
-        <x:v>개발 fixture 5종 재생</x:v>
+        <x:v>대체 fixture 5종 저장 전후 대조</x:v>
       </x:c>
       <x:c r="E20" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F20" s="33" t="str">
-        <x:v>운영 실패 5종 모두 마지막 정상값 421.6 유지</x:v>
+        <x:v>5종 모두 D1-B 421.6·관측 시각·일별 1건 보존</x:v>
       </x:c>
       <x:c r="G20" s="33" t="str">
-        <x:v>Vercel /api/lab 실패 5종</x:v>
+        <x:v>lib/synthetic.test.ts, ALT-T04-COSMIC-PULSE-V1</x:v>
       </x:c>
       <x:c r="H20" s="33" t="str">
-        <x:v>공식 T04 asset으로 최종 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I20" s="1"/>
       <x:c r="J20" s="1"/>
@@ -2599,7 +2599,7 @@
       <x:c r="M20" s="1"/>
       <x:c r="N20" s="1"/>
     </x:row>
-    <x:row r="21" ht="48" customHeight="1">
+    <x:row r="21" ht="58" customHeight="1">
       <x:c r="A21" s="32" t="str">
         <x:v>T04-C18</x:v>
       </x:c>
@@ -2610,19 +2610,19 @@
         <x:v>실패 뒤 마지막 정상값에 오래된 값 표시가 붙는다.</x:v>
       </x:c>
       <x:c r="D21" s="33" t="str">
-        <x:v>개발 fixture 5종 상태 확인</x:v>
+        <x:v>대체 fixture 5종 상태 확인</x:v>
       </x:c>
       <x:c r="E21" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F21" s="33" t="str">
-        <x:v>운영 실패 5종 모두 stale 상태 표시</x:v>
+        <x:v>5종 모두 stale 및 실패 코드별 다음 행동 표시</x:v>
       </x:c>
       <x:c r="G21" s="33" t="str">
-        <x:v>Vercel /api/lab 실패 5종</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab</x:v>
       </x:c>
       <x:c r="H21" s="33" t="str">
-        <x:v>공식 T04 asset으로 최종 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I21" s="1"/>
       <x:c r="J21" s="1"/>
@@ -2631,7 +2631,7 @@
       <x:c r="M21" s="1"/>
       <x:c r="N21" s="1"/>
     </x:row>
-    <x:row r="22" ht="48" customHeight="1">
+    <x:row r="22" ht="58" customHeight="1">
       <x:c r="A22" s="32" t="str">
         <x:v>T04-C19</x:v>
       </x:c>
@@ -2642,19 +2642,19 @@
         <x:v>재시도 행동과 공식 T04-RECOVER-D2 복구 결과를 확인한다.</x:v>
       </x:c>
       <x:c r="D22" s="33" t="str">
-        <x:v>DEV-RECOVER-D2 재생</x:v>
+        <x:v>ALT-T04-RECOVER-D2 재생·중복 실행</x:v>
       </x:c>
       <x:c r="E22" s="36" t="str">
-        <x:v>부분 충족</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F22" s="33" t="str">
-        <x:v>운영 DEV-RECOVER-D2: fresh / error none / 일별 2건</x:v>
+        <x:v>fresh / none / 1→2 / +1, D2 재실행 후에도 2건</x:v>
       </x:c>
       <x:c r="G22" s="33" t="str">
-        <x:v>Vercel /api/lab</x:v>
+        <x:v>https://real-info-board.vercel.app/lab, /api/lab, ALT-T04-COSMIC-PULSE-V1</x:v>
       </x:c>
       <x:c r="H22" s="33" t="str">
-        <x:v>공식 T04-RECOVER-D2 확보 후 재검증</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I22" s="1"/>
       <x:c r="J22" s="1"/>
@@ -2872,13 +2872,13 @@
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F29" s="33" t="str">
-        <x:v>DEV-* 값만 사용하며 실제 SQLite에 쓰지 않음</x:v>
+        <x:v>합성값은 요청별 in_memory 저장소만 사용하며 Supabase·SQLite에 기록하지 않음</x:v>
       </x:c>
       <x:c r="G29" s="33" t="str">
-        <x:v>lib/synthetic.ts, /lab</x:v>
+        <x:v>lib/synthetic.ts, public-contract.json, https://real-info-board.vercel.app/lab</x:v>
       </x:c>
       <x:c r="H29" s="33" t="str">
-        <x:v>공식 asset도 실제 저장과 격리</x:v>
+        <x:v>없음</x:v>
       </x:c>
       <x:c r="I29" s="1"/>
       <x:c r="J29" s="1"/>
@@ -5271,7 +5271,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="27" t="str">
-        <x:v>실행일 2026-09-10 KST · 환경: Vercel / Next.js 16.3.4 / Supabase · 코드 commit e94657a</x:v>
+        <x:v>실행일 2026-09-10 KST · 환경: Vercel / Next.js 16.3.4 / Supabase · 코드 commit fe64094</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -5382,13 +5382,13 @@
         <x:v>전체 통과</x:v>
       </x:c>
       <x:c r="D7" s="49" t="str">
-        <x:v>7 files / 15 tests passed</x:v>
+        <x:v>7 files / 16 tests passed</x:v>
       </x:c>
       <x:c r="E7" s="49" t="str">
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F7" s="49" t="str">
-        <x:v>Vitest 5.0.0 · 0.94s</x:v>
+        <x:v>Vitest 5.0.0 · 4.14s</x:v>
       </x:c>
       <x:c r="G7" s="1"/>
       <x:c r="H7" s="1"/>
@@ -5410,13 +5410,13 @@
         <x:v>빌드 성공</x:v>
       </x:c>
       <x:c r="D8" s="49" t="str">
-        <x:v>Vercel build 성공 / 7개 route</x:v>
+        <x:v>Vercel production build 성공 / 7개 route</x:v>
       </x:c>
       <x:c r="E8" s="49" t="str">
         <x:v>통과</x:v>
       </x:c>
       <x:c r="F8" s="49" t="str">
-        <x:v>Next.js 16.3.4 · compile 0.82s</x:v>
+        <x:v>Next.js 16.3.4</x:v>
       </x:c>
       <x:c r="G8" s="1"/>
       <x:c r="H8" s="1"/>
@@ -5572,19 +5572,19 @@
         <x:v>느린 응답</x:v>
       </x:c>
       <x:c r="B14" s="49" t="str">
-        <x:v>DEV-SLOW</x:v>
+        <x:v>ALT-T04-SLOW</x:v>
       </x:c>
       <x:c r="C14" s="49" t="str">
-        <x:v>stale / slow_response</x:v>
+        <x:v>격리 adapter 재생</x:v>
       </x:c>
       <x:c r="D14" s="49" t="str">
-        <x:v>421.6 유지 / 재시도 안내</x:v>
+        <x:v>421.6 / stale / slow_response / 1→1 / +0 / 보존</x:v>
       </x:c>
       <x:c r="E14" s="49" t="str">
-        <x:v>운영 통과</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F14" s="49" t="str">
-        <x:v>Vercel /api/lab</x:v>
+        <x:v>Vercel /api/lab · in_memory</x:v>
       </x:c>
       <x:c r="G14" s="1"/>
       <x:c r="H14" s="1"/>
@@ -5600,19 +5600,19 @@
         <x:v>접근 거절</x:v>
       </x:c>
       <x:c r="B15" s="49" t="str">
-        <x:v>DEV-DENIED</x:v>
+        <x:v>ALT-T04-DENIED</x:v>
       </x:c>
       <x:c r="C15" s="49" t="str">
-        <x:v>stale / upstream_denied</x:v>
+        <x:v>격리 adapter 재생</x:v>
       </x:c>
       <x:c r="D15" s="49" t="str">
-        <x:v>421.6 유지 / 원천 확인 안내</x:v>
+        <x:v>421.6 / stale / upstream_denied / 1→1 / +0 / 보존</x:v>
       </x:c>
       <x:c r="E15" s="49" t="str">
-        <x:v>운영 통과</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F15" s="49" t="str">
-        <x:v>Vercel /api/lab</x:v>
+        <x:v>Vercel /api/lab · in_memory</x:v>
       </x:c>
       <x:c r="G15" s="1"/>
       <x:c r="H15" s="1"/>
@@ -5628,19 +5628,19 @@
         <x:v>호출 제한</x:v>
       </x:c>
       <x:c r="B16" s="49" t="str">
-        <x:v>DEV-RATE-LIMIT</x:v>
+        <x:v>ALT-T04-RATE-LIMIT</x:v>
       </x:c>
       <x:c r="C16" s="49" t="str">
-        <x:v>stale / rate_limited</x:v>
+        <x:v>격리 adapter 재생</x:v>
       </x:c>
       <x:c r="D16" s="49" t="str">
-        <x:v>421.6 유지 / 대기 안내</x:v>
+        <x:v>421.6 / stale / rate_limited / 1→1 / +0 / 보존</x:v>
       </x:c>
       <x:c r="E16" s="49" t="str">
-        <x:v>운영 통과</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F16" s="49" t="str">
-        <x:v>Vercel /api/lab</x:v>
+        <x:v>Vercel /api/lab · in_memory</x:v>
       </x:c>
       <x:c r="G16" s="1"/>
       <x:c r="H16" s="1"/>
@@ -5656,19 +5656,19 @@
         <x:v>오프라인</x:v>
       </x:c>
       <x:c r="B17" s="49" t="str">
-        <x:v>DEV-OFFLINE</x:v>
+        <x:v>ALT-T04-OFFLINE</x:v>
       </x:c>
       <x:c r="C17" s="49" t="str">
-        <x:v>stale / offline</x:v>
+        <x:v>격리 adapter 재생</x:v>
       </x:c>
       <x:c r="D17" s="49" t="str">
-        <x:v>421.6 유지 / 연결 확인 안내</x:v>
+        <x:v>421.6 / stale / offline / 1→1 / +0 / 보존</x:v>
       </x:c>
       <x:c r="E17" s="49" t="str">
-        <x:v>운영 통과</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F17" s="49" t="str">
-        <x:v>Vercel /api/lab</x:v>
+        <x:v>Vercel /api/lab · in_memory</x:v>
       </x:c>
       <x:c r="G17" s="1"/>
       <x:c r="H17" s="1"/>
@@ -5684,19 +5684,19 @@
         <x:v>형식 변경</x:v>
       </x:c>
       <x:c r="B18" s="49" t="str">
-        <x:v>DEV-FORMAT</x:v>
+        <x:v>ALT-T04-FORMAT</x:v>
       </x:c>
       <x:c r="C18" s="49" t="str">
-        <x:v>stale / format_changed</x:v>
+        <x:v>격리 adapter 재생</x:v>
       </x:c>
       <x:c r="D18" s="49" t="str">
-        <x:v>421.6 유지 / 어댑터 점검</x:v>
+        <x:v>421.6 / stale / format_changed / 1→1 / +0 / 보존</x:v>
       </x:c>
       <x:c r="E18" s="49" t="str">
-        <x:v>운영 통과</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F18" s="49" t="str">
-        <x:v>Vercel /api/lab</x:v>
+        <x:v>Vercel /api/lab · in_memory</x:v>
       </x:c>
       <x:c r="G18" s="1"/>
       <x:c r="H18" s="1"/>
@@ -5712,19 +5712,19 @@
         <x:v>복구</x:v>
       </x:c>
       <x:c r="B19" s="50" t="str">
-        <x:v>DEV-RECOVER-D2</x:v>
+        <x:v>ALT-T04-RECOVER-D2</x:v>
       </x:c>
       <x:c r="C19" s="50" t="str">
-        <x:v>fresh / none / 2건</x:v>
+        <x:v>격리 adapter 재생</x:v>
       </x:c>
       <x:c r="D19" s="50" t="str">
-        <x:v>447.2 / fresh / error none / 2건</x:v>
+        <x:v>447.2 / fresh / none / 1→2 / +1 / 중복 후 2건</x:v>
       </x:c>
       <x:c r="E19" s="50" t="str">
-        <x:v>운영 통과</x:v>
+        <x:v>통과</x:v>
       </x:c>
       <x:c r="F19" s="50" t="str">
-        <x:v>Vercel /api/lab</x:v>
+        <x:v>Vercel /api/lab · in_memory</x:v>
       </x:c>
       <x:c r="G19" s="1"/>
       <x:c r="H19" s="1"/>
@@ -5898,10 +5898,10 @@
       <x:c r="B27" s="1" t="str">
         <x:v>https://real-info-board.vercel.app</x:v>
       </x:c>
-      <x:c r="C27" s="1"/>
-      <x:c r="D27" s="1"/>
-      <x:c r="E27" s="1"/>
-      <x:c r="F27" s="1"/>
+      <x:c r="C27" s="1" t="str"/>
+      <x:c r="D27" s="1" t="str"/>
+      <x:c r="E27" s="1" t="str"/>
+      <x:c r="F27" s="1" t="str"/>
       <x:c r="G27" s="1"/>
       <x:c r="H27" s="1"/>
       <x:c r="I27" s="1"/>
@@ -5911,17 +5911,25 @@
       <x:c r="M27" s="1"/>
       <x:c r="N27" s="1"/>
     </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="25" t="str">
-        <x:v>공식 T04 시험 asset</x:v>
-      </x:c>
-      <x:c r="B28" s="25" t="str">
-        <x:v>미제공: assets/studio-task-assets/t04-real-information-board/</x:v>
-      </x:c>
-      <x:c r="C28" s="1"/>
-      <x:c r="D28" s="1"/>
-      <x:c r="E28" s="1"/>
-      <x:c r="F28" s="1"/>
+    <x:row r="28" ht="72" customHeight="1">
+      <x:c r="A28" s="50" t="str">
+        <x:v>승인 대체 T04 package</x:v>
+      </x:c>
+      <x:c r="B28" s="50" t="str">
+        <x:v>ALT-T04-COSMIC-PULSE-V1 · assets/studio-task-assets/t04-real-information-board/</x:v>
+      </x:c>
+      <x:c r="C28" s="49" t="str">
+        <x:v>README SHA-256 5df7886b5d7669110708c2dde36a1c04683d679c84c64e72fa84899864b07356</x:v>
+      </x:c>
+      <x:c r="D28" s="49" t="str">
+        <x:v>contract SHA-256 b90c8ea8b6a0b86119a8f86261d51c58a66463b79b0bbcecbd26e72d89f1f020</x:v>
+      </x:c>
+      <x:c r="E28" s="49" t="str">
+        <x:v>manifest 자동 검증 통과</x:v>
+      </x:c>
+      <x:c r="F28" s="49" t="str">
+        <x:v>https://github.com/hyeseong-dev/real_info_board</x:v>
+      </x:c>
       <x:c r="G28" s="1"/>
       <x:c r="H28" s="1"/>
       <x:c r="I28" s="1"/>

</xml_diff>